<commit_message>
- Bug fix sort and filter - Update search list view
</commit_message>
<xml_diff>
--- a/app/views/Reports/households.xlsx
+++ b/app/views/Reports/households.xlsx
@@ -6,14 +6,14 @@
     <sheet state="visible" name="Residents" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">Residents!$B$2:$U$5</definedName>
+    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">Residents!$B$2:$T$5</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
   <si>
     <t>id</t>
   </si>
@@ -25,9 +25,6 @@
   </si>
   <si>
     <t>barangay</t>
-  </si>
-  <si>
-    <t>barangayno</t>
   </si>
   <si>
     <t>rmflrblockno</t>
@@ -84,14 +81,16 @@
   <si>
     <r>
       <rPr>
-        <rFont val="Calibri"/>
+        <rFont val="Calibri, Arial"/>
+        <color rgb="FF0563C1"/>
         <sz val="11.0"/>
+        <u/>
       </rPr>
       <t>${</t>
     </r>
     <r>
       <rPr>
-        <rFont val="Calibri"/>
+        <rFont val="Calibri, Arial"/>
         <color rgb="FF1155CC"/>
         <sz val="11.0"/>
         <u/>
@@ -100,89 +99,67 @@
     </r>
     <r>
       <rPr>
-        <rFont val="Calibri"/>
+        <rFont val="Calibri, Arial"/>
+        <color rgb="FF0563C1"/>
         <sz val="11.0"/>
+        <u/>
       </rPr>
       <t>}</t>
     </r>
   </si>
   <si>
-    <t>KALINGA</t>
-  </si>
-  <si>
-    <t>TABUK CITY</t>
+    <t>${record.province}</t>
+  </si>
+  <si>
+    <t>${record.municipality}</t>
   </si>
   <si>
     <t>${record.barangay}</t>
   </si>
   <si>
-    <t>${record.getAddress()}</t>
-  </si>
-  <si>
-    <t>${record.getHouseNo()}</t>
-  </si>
-  <si>
-    <t>${record.getStreet()}</t>
-  </si>
-  <si>
-    <t>${record.getHead()}</t>
-  </si>
-  <si>
-    <t>${record.getTotalNumber()}</t>
-  </si>
-  <si>
-    <t>${record.getHouseOwnership()}</t>
-  </si>
-  <si>
-    <t>${record.getLotOwnership()}</t>
-  </si>
-  <si>
-    <t>${record.getLighting()}</t>
-  </si>
-  <si>
-    <t>${record.getCooking()}</t>
-  </si>
-  <si>
-    <t>${record.getWaterSource()}</t>
-  </si>
-  <si>
-    <t>${record.getGarbageDisposal()}</t>
-  </si>
-  <si>
-    <t>${record.getHasTrashSegregation()}</t>
-  </si>
-  <si>
-    <t>${record.getToiletFacility()}</t>
-  </si>
-  <si>
-    <t>${record.getBuildingType()}</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color rgb="FF000000"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>${record.getB</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color rgb="FF000000"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>u</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color rgb="FF000000"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>ildingMaterial()}</t>
-    </r>
+    <t>${record.blockNo}</t>
+  </si>
+  <si>
+    <t>${record.houseNo}</t>
+  </si>
+  <si>
+    <t>${record.street}</t>
+  </si>
+  <si>
+    <t>${record.head}</t>
+  </si>
+  <si>
+    <t>${record.totalNo}</t>
+  </si>
+  <si>
+    <t>${record.houseOwnership}</t>
+  </si>
+  <si>
+    <t>${record.lotOwnership}</t>
+  </si>
+  <si>
+    <t>${record.lighting}</t>
+  </si>
+  <si>
+    <t>${record.cooking}</t>
+  </si>
+  <si>
+    <t>${record.waterSource}</t>
+  </si>
+  <si>
+    <t>${record.garbageDisposal}</t>
+  </si>
+  <si>
+    <t>${record.hasTrashSegregation}</t>
+  </si>
+  <si>
+    <t>${record.toiletFacility}</t>
+  </si>
+  <si>
+    <t>${record.buildingType}</t>
+  </si>
+  <si>
+    <t>${record.buildingMaterial}</t>
   </si>
   <si>
     <t>&lt;/jx:forEach&gt;</t>
@@ -195,11 +172,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy/mm/dd\ h:mm:ss\ AM/PM"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11.0"/>
@@ -220,12 +198,7 @@
     <font>
       <u/>
       <sz val="11.0"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11.0"/>
-      <color rgb="FF000000"/>
+      <color rgb="FF0563C1"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -261,8 +234,19 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="3">
     <border/>
+    <border>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
@@ -277,35 +261,11 @@
         <color rgb="FF000000"/>
       </bottom>
     </border>
-    <border>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
-    <border>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-    </border>
-    <border>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="19">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -320,46 +280,44 @@
     <xf borderId="0" fillId="2" fontId="2" numFmtId="49" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
     <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="2" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="2" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="0"/>
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="2" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment vertical="bottom"/>
     </xf>
     <xf borderId="2" fillId="2" fontId="2" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
+      <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
+    <xf borderId="2" fillId="0" fontId="2" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment vertical="bottom"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="4" fillId="2" fontId="2" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
+      <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -572,28 +530,28 @@
   <sheetPr>
     <pageSetUpPr/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
+  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="4.0"/>
-    <col customWidth="1" min="2" max="2" width="14.63"/>
-    <col customWidth="1" min="3" max="3" width="7.63"/>
-    <col customWidth="1" min="4" max="4" width="13.38"/>
-    <col customWidth="1" min="5" max="5" width="17.38"/>
-    <col customWidth="1" min="6" max="6" width="9.88"/>
-    <col customWidth="1" min="7" max="7" width="10.88"/>
-    <col customWidth="1" min="8" max="8" width="11.88"/>
-    <col customWidth="1" min="9" max="9" width="15.88"/>
-    <col customWidth="1" min="10" max="10" width="23.25"/>
-    <col customWidth="1" min="11" max="11" width="18.25"/>
-    <col customWidth="1" min="12" max="12" width="25.88"/>
-    <col customWidth="1" min="13" max="13" width="24.75"/>
-    <col customWidth="1" min="14" max="14" width="25.13"/>
-    <col customWidth="1" min="15" max="15" width="23.38"/>
-    <col customWidth="1" min="16" max="16" width="23.25"/>
-    <col customWidth="1" min="17" max="18" width="23.5"/>
-    <col customWidth="1" min="19" max="19" width="24.13"/>
-    <col customWidth="1" min="20" max="20" width="28.0"/>
-    <col customWidth="1" min="21" max="21" width="26.63"/>
+    <col customWidth="1" min="1" max="1" width="4.57"/>
+    <col customWidth="1" min="2" max="2" width="12.86"/>
+    <col customWidth="1" min="3" max="3" width="19.86"/>
+    <col customWidth="1" min="4" max="4" width="21.43"/>
+    <col customWidth="1" min="5" max="5" width="22.57"/>
+    <col customWidth="1" min="6" max="6" width="16.86"/>
+    <col customWidth="1" min="7" max="7" width="15.71"/>
+    <col customWidth="1" min="8" max="8" width="19.0"/>
+    <col customWidth="1" min="9" max="9" width="18.29"/>
+    <col customWidth="1" min="10" max="10" width="8.71"/>
+    <col customWidth="1" min="11" max="11" width="22.14"/>
+    <col customWidth="1" min="12" max="12" width="23.71"/>
+    <col customWidth="1" min="13" max="13" width="18.14"/>
+    <col customWidth="1" min="14" max="14" width="26.86"/>
+    <col customWidth="1" min="15" max="15" width="26.57"/>
+    <col customWidth="1" min="16" max="16" width="23.86"/>
+    <col customWidth="1" min="17" max="17" width="17.14"/>
+    <col customWidth="1" min="18" max="18" width="24.0"/>
+    <col customWidth="1" min="19" max="19" width="24.29"/>
+    <col customWidth="1" min="20" max="20" width="25.43"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customHeight="1">
@@ -601,127 +559,124 @@
       <c r="B1" s="1"/>
       <c r="C1" s="2"/>
       <c r="D1" s="3"/>
-      <c r="E1" s="4"/>
+      <c r="E1" s="3"/>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
       <c r="I1" s="4"/>
-      <c r="J1" s="5"/>
+      <c r="J1" s="4"/>
       <c r="K1" s="4"/>
       <c r="L1" s="4"/>
       <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
+      <c r="N1" s="5"/>
+      <c r="O1" s="5"/>
       <c r="P1" s="4"/>
-      <c r="Q1" s="4"/>
-      <c r="R1" s="4"/>
-      <c r="S1" s="4"/>
-      <c r="T1" s="4"/>
-      <c r="U1" s="4"/>
+      <c r="Q1" s="6"/>
+      <c r="R1" s="6"/>
+      <c r="S1" s="6"/>
+      <c r="T1" s="6"/>
     </row>
     <row r="2" ht="48.0" customHeight="1">
-      <c r="A2" s="1"/>
-      <c r="B2" s="6" t="s">
+      <c r="A2" s="7"/>
+      <c r="B2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="G2" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="H2" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="I2" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="7" t="s">
+      <c r="J2" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="K2" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="L2" s="8" t="s">
+      <c r="L2" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="M2" s="8" t="s">
+      <c r="M2" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="N2" s="8" t="s">
+      <c r="N2" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="O2" s="8" t="s">
+      <c r="O2" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="P2" s="8" t="s">
+      <c r="P2" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="Q2" s="8" t="s">
+      <c r="Q2" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="R2" s="8" t="s">
+      <c r="R2" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="S2" s="8" t="s">
+      <c r="S2" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="T2" s="8" t="s">
+      <c r="T2" s="10" t="s">
         <v>18</v>
-      </c>
-      <c r="U2" s="8" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="3" ht="18.75" customHeight="1">
-      <c r="A3" s="1"/>
-      <c r="B3" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="10"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="12"/>
+      <c r="A3" s="7"/>
+      <c r="B3" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="12"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
       <c r="F3" s="12"/>
       <c r="G3" s="12"/>
       <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="13"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="12"/>
       <c r="K3" s="12"/>
       <c r="L3" s="12"/>
       <c r="M3" s="12"/>
-      <c r="N3" s="12"/>
-      <c r="O3" s="12"/>
+      <c r="N3" s="15"/>
+      <c r="O3" s="15"/>
       <c r="P3" s="12"/>
       <c r="Q3" s="12"/>
-      <c r="R3" s="14"/>
+      <c r="R3" s="12"/>
       <c r="S3" s="12"/>
       <c r="T3" s="12"/>
-      <c r="U3" s="12"/>
     </row>
     <row r="4">
-      <c r="A4" s="4"/>
-      <c r="B4" s="15" t="s">
+      <c r="A4" s="7"/>
+      <c r="B4" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="D4" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="E4" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="F4" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="F4" s="16"/>
       <c r="G4" s="17" t="s">
         <v>25</v>
       </c>
@@ -737,61 +692,57 @@
       <c r="K4" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="L4" s="17" t="s">
+      <c r="L4" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="M4" s="18" t="s">
+      <c r="M4" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="N4" s="17" t="s">
+      <c r="N4" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="O4" s="18" t="s">
+      <c r="O4" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="P4" s="18" t="s">
+      <c r="P4" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="Q4" s="18" t="s">
+      <c r="Q4" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="R4" s="18" t="s">
+      <c r="R4" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="S4" s="18" t="s">
+      <c r="S4" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="T4" s="17" t="s">
+      <c r="T4" s="12" t="s">
         <v>38</v>
-      </c>
-      <c r="U4" s="18" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2"/>
-      <c r="B5" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="C5" s="10"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="19"/>
-      <c r="G5" s="19"/>
-      <c r="H5" s="19"/>
-      <c r="I5" s="19"/>
-      <c r="J5" s="20"/>
-      <c r="K5" s="19"/>
-      <c r="L5" s="19"/>
-      <c r="M5" s="19"/>
-      <c r="N5" s="19"/>
-      <c r="O5" s="19"/>
-      <c r="P5" s="19"/>
-      <c r="Q5" s="19"/>
-      <c r="R5" s="14"/>
-      <c r="S5" s="19"/>
-      <c r="T5" s="19"/>
-      <c r="U5" s="19"/>
+      <c r="A5" s="7"/>
+      <c r="B5" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" s="12"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="12"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="12"/>
+      <c r="K5" s="12"/>
+      <c r="L5" s="12"/>
+      <c r="M5" s="12"/>
+      <c r="N5" s="15"/>
+      <c r="O5" s="15"/>
+      <c r="P5" s="12"/>
+      <c r="Q5" s="12"/>
+      <c r="R5" s="12"/>
+      <c r="S5" s="12"/>
+      <c r="T5" s="12"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -1774,7 +1725,7 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="$B$2:$U$5"/>
+  <autoFilter ref="$B$2:$T$5"/>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="B4"/>
   </hyperlinks>

</xml_diff>